<commit_message>
Jury: Adjust TO section
</commit_message>
<xml_diff>
--- a/local/templates/jury/JurySheet.xlsx
+++ b/local/templates/jury/JurySheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/jury/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/templates/jury/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{451CFEFD-27F5-8945-A4C7-AD9484B8E2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57954C36-FE68-0F45-B5CE-C2D4380E4A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8660" yWindow="500" windowWidth="32300" windowHeight="23500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8660" yWindow="660" windowWidth="32300" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jury" sheetId="1" r:id="rId1"/>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -170,15 +170,6 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Speaker</t>
-  </si>
-  <si>
-    <t>Timekeeper</t>
-  </si>
-  <si>
-    <t>Technical Controller</t>
-  </si>
-  <si>
     <t>${athlete.entryTotal}</t>
   </si>
   <si>
@@ -269,19 +260,16 @@
     <t>Center</t>
   </si>
   <si>
-    <t>Marshal</t>
-  </si>
-  <si>
     <t>Referees</t>
   </si>
   <si>
-    <t>Signature</t>
-  </si>
-  <si>
     <t>Session ${session.name} - ${session.ageGroupInfo.0.formattedRange}</t>
   </si>
   <si>
-    <t xml:space="preserve">Jury President Signature  </t>
+    <t>Initials</t>
+  </si>
+  <si>
+    <t>Jury President Signature</t>
   </si>
 </sst>
 </file>
@@ -512,7 +500,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -547,13 +535,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -622,8 +603,6 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -648,6 +627,26 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
@@ -670,27 +669,15 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -699,23 +686,8 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Emphase 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1427,66 +1399,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
+      <c r="R1" s="47"/>
+      <c r="S1" s="47"/>
+      <c r="T1" s="47"/>
+      <c r="U1" s="47"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="47"/>
     </row>
     <row r="2" spans="1:27" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
+      <c r="A2" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
       <c r="Q2" s="3"/>
-      <c r="R2" s="46" t="s">
-        <v>29</v>
-      </c>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="15"/>
+      <c r="R2" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="S2" s="48"/>
+      <c r="T2" s="48"/>
+      <c r="U2" s="48"/>
+      <c r="V2" s="12"/>
       <c r="W2" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
-      <c r="B3" s="15"/>
+      <c r="B3" s="12"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -1498,22 +1470,22 @@
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
       <c r="T3" s="3"/>
-      <c r="U3" s="15"/>
-      <c r="V3" s="15"/>
-      <c r="W3" s="15"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
     </row>
     <row r="4" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="18"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="3"/>
       <c r="C4" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -1524,87 +1496,87 @@
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
       <c r="L4" s="5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="58" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" s="59"/>
-      <c r="P4" s="59"/>
-      <c r="Q4" s="59"/>
-      <c r="R4" s="58" t="s">
-        <v>31</v>
-      </c>
-      <c r="S4" s="59"/>
-      <c r="T4" s="59"/>
-      <c r="U4" s="59"/>
-      <c r="V4" s="52"/>
-      <c r="W4" s="53"/>
+        <v>19</v>
+      </c>
+      <c r="N4" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="57"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="57"/>
+      <c r="R4" s="56" t="s">
+        <v>28</v>
+      </c>
+      <c r="S4" s="57"/>
+      <c r="T4" s="57"/>
+      <c r="U4" s="57"/>
+      <c r="V4" s="53"/>
+      <c r="W4" s="54"/>
     </row>
     <row r="5" spans="1:27" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="F5" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="50" t="s">
+      <c r="L5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
-      <c r="J5" s="50"/>
-      <c r="K5" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="M5" s="19" t="s">
+      <c r="M5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="N5" s="42">
+      <c r="N5" s="37">
         <v>1</v>
       </c>
-      <c r="O5" s="38">
+      <c r="O5" s="33">
         <v>2</v>
       </c>
-      <c r="P5" s="38">
+      <c r="P5" s="33">
         <v>3</v>
       </c>
-      <c r="Q5" s="38" t="s">
+      <c r="Q5" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="R5" s="42">
+      <c r="R5" s="37">
         <v>1</v>
       </c>
-      <c r="S5" s="38">
+      <c r="S5" s="33">
         <v>2</v>
       </c>
-      <c r="T5" s="38">
+      <c r="T5" s="33">
         <v>3</v>
       </c>
-      <c r="U5" s="38" t="s">
+      <c r="U5" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="V5" s="43" t="s">
+      <c r="V5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="W5" s="44" t="s">
-        <v>23</v>
+      <c r="W5" s="39" t="s">
+        <v>20</v>
       </c>
       <c r="X5"/>
       <c r="Y5"/>
@@ -1612,45 +1584,45 @@
       <c r="AA5"/>
     </row>
     <row r="6" spans="1:27" s="6" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="25" t="s">
+      <c r="A6" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="L6" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
+      <c r="M6" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
       <c r="V6" s="8"/>
       <c r="W6" s="8"/>
       <c r="X6"/>
@@ -1659,290 +1631,249 @@
       <c r="AA6"/>
     </row>
     <row r="7" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="57" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="57"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="39" t="s">
+      <c r="A7" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="55"/>
+      <c r="C7" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="44"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="15"/>
-      <c r="O7" s="15"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
-      <c r="S7" s="28"/>
-      <c r="T7" s="30"/>
-      <c r="U7" s="30"/>
-      <c r="V7" s="31"/>
-      <c r="W7" s="15"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="S7" s="25"/>
+      <c r="T7" s="27"/>
+      <c r="U7" s="27"/>
+      <c r="V7" s="28"/>
+      <c r="W7" s="12"/>
     </row>
     <row r="8" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="54" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
+      <c r="A8" s="59"/>
+      <c r="C8" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="42"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="11"/>
-      <c r="G8" s="22"/>
+      <c r="G8" s="11"/>
       <c r="H8" s="11"/>
-      <c r="I8" s="22"/>
+      <c r="I8" s="19"/>
       <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
+      <c r="K8" s="19"/>
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="R8" s="36"/>
-      <c r="S8" s="36"/>
-      <c r="T8" s="36"/>
-      <c r="U8" s="36"/>
-      <c r="V8" s="36"/>
-      <c r="W8" s="36"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="S8" s="31"/>
+      <c r="T8" s="31"/>
+      <c r="U8" s="31"/>
+      <c r="V8" s="31"/>
+      <c r="W8" s="31"/>
     </row>
     <row r="9" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="55" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="55"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="58"/>
+      <c r="C9" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="32"/>
+      <c r="E9" s="7"/>
       <c r="F9" s="9"/>
-      <c r="G9" s="22"/>
+      <c r="G9" s="9"/>
       <c r="H9" s="9"/>
-      <c r="I9" s="22"/>
+      <c r="I9" s="19"/>
       <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="R9" s="37"/>
-      <c r="S9" s="37"/>
-      <c r="T9" s="37"/>
-      <c r="U9" s="37"/>
-      <c r="V9" s="37"/>
-      <c r="W9" s="37"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45"/>
+      <c r="P9" s="46"/>
+      <c r="Q9" s="46"/>
+      <c r="S9" s="31"/>
+      <c r="T9" s="31"/>
+      <c r="U9" s="31"/>
+      <c r="V9" s="31"/>
+      <c r="W9" s="31"/>
     </row>
     <row r="10" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="35"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
+      <c r="A10" s="58"/>
+      <c r="C10" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="32"/>
+      <c r="E10" s="7"/>
       <c r="F10" s="9"/>
-      <c r="G10" s="22"/>
+      <c r="G10" s="9"/>
       <c r="H10" s="9"/>
-      <c r="I10" s="22"/>
+      <c r="I10" s="19"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="R10" s="37"/>
-      <c r="S10" s="37"/>
-      <c r="T10" s="37"/>
-      <c r="U10" s="37"/>
-      <c r="V10" s="37"/>
-      <c r="W10" s="37"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="29"/>
+      <c r="S10" s="31"/>
+      <c r="T10" s="31"/>
+      <c r="U10" s="31"/>
+      <c r="V10" s="31"/>
+      <c r="W10" s="31"/>
     </row>
     <row r="11" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="56" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="56"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="R11" s="37"/>
-      <c r="S11" s="37"/>
-      <c r="T11" s="37"/>
-      <c r="U11" s="37"/>
-      <c r="V11" s="37"/>
-      <c r="W11" s="37"/>
+      <c r="C11" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="43"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="12"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="31"/>
     </row>
     <row r="12" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="54"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="42"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="11"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="34"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="R12" s="37"/>
-      <c r="S12" s="37"/>
-      <c r="T12" s="37"/>
-      <c r="U12" s="37"/>
-      <c r="V12" s="37"/>
-      <c r="W12" s="37"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="31"/>
+      <c r="S12" s="31"/>
+      <c r="T12" s="31"/>
+      <c r="U12" s="31"/>
+      <c r="V12" s="31"/>
+      <c r="W12" s="31"/>
     </row>
     <row r="13" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
+      <c r="C13" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="35"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="9"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="30"/>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="51"/>
-      <c r="S13" s="51"/>
-      <c r="T13" s="32"/>
-      <c r="U13" s="31"/>
-      <c r="V13" s="22"/>
-      <c r="W13" s="15"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="12"/>
+      <c r="S13" s="25"/>
+      <c r="T13" s="29"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="12"/>
     </row>
     <row r="14" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+      <c r="C14" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="35"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="15"/>
-      <c r="S14" s="15"/>
-      <c r="T14" s="15"/>
-      <c r="U14" s="15"/>
-      <c r="V14" s="15"/>
-      <c r="W14" s="15"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
     </row>
     <row r="15" spans="1:27" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="65"/>
-      <c r="B15" s="65"/>
-      <c r="C15" s="66"/>
-      <c r="D15" s="66"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="66"/>
+      <c r="A15" s="41"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J15" s="60"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="61"/>
-      <c r="O15" s="61"/>
-      <c r="P15" s="15"/>
+      <c r="I15" s="3"/>
+      <c r="P15" s="12"/>
       <c r="Q15" s="5"/>
-      <c r="R15" s="15"/>
-      <c r="S15" s="15"/>
-      <c r="T15" s="15"/>
-      <c r="U15" s="15"/>
-      <c r="V15" s="15"/>
-      <c r="W15" s="15"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="12"/>
     </row>
     <row r="16" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="33"/>
-      <c r="B16" s="33"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="30"/>
     </row>
-    <row r="17" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I17" s="62"/>
-      <c r="J17" s="63"/>
-      <c r="K17" s="63"/>
-      <c r="L17" s="63"/>
-      <c r="M17" s="63"/>
-      <c r="N17" s="64"/>
-      <c r="O17" s="64"/>
+    <row r="17" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I17" s="40"/>
     </row>
-    <row r="18" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="9:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="9:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1979,20 +1910,15 @@
     <row r="66" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="13">
+  <mergeCells count="8">
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="R2:U2"/>
     <mergeCell ref="F6:J6"/>
     <mergeCell ref="F5:J5"/>
-    <mergeCell ref="R13:S13"/>
     <mergeCell ref="V4:W4"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A7:B7"/>
     <mergeCell ref="N4:Q4"/>
     <mergeCell ref="R4:U4"/>
+    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:F6 K6:M6">
     <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">

</xml_diff>